<commit_message>
Fix owner account creation: lower password min length to 8 and add gymName to registration form
</commit_message>
<xml_diff>
--- a/gym_platform_development_only_tracker.xlsx
+++ b/gym_platform_development_only_tracker.xlsx
@@ -1926,6 +1926,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="34" customHeight="1">
       <c r="A49" s="34" t="inlineStr">
@@ -1953,6 +1958,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="34" customHeight="1">
       <c r="A50" s="34" t="inlineStr">
@@ -1980,6 +1990,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="34" customHeight="1">
       <c r="A51" s="34" t="inlineStr">
@@ -2007,6 +2022,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="34" customHeight="1">
       <c r="A52" s="34" t="inlineStr">
@@ -2034,6 +2054,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="34" customHeight="1">
       <c r="A53" s="34" t="inlineStr">
@@ -2061,6 +2086,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="34" customHeight="1">
       <c r="A54" s="34" t="inlineStr">
@@ -2088,6 +2118,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="34" customHeight="1">
       <c r="A55" s="34" t="inlineStr">
@@ -2115,6 +2150,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="34" customHeight="1">
       <c r="A56" s="34" t="inlineStr">
@@ -2142,6 +2182,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="34" customHeight="1">
       <c r="A57" s="34" t="inlineStr">
@@ -2169,6 +2214,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="34" customHeight="1">
       <c r="A58" s="34" t="inlineStr">
@@ -2196,6 +2246,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="34" customHeight="1">
       <c r="A59" s="34" t="inlineStr">
@@ -2223,6 +2278,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="34" customHeight="1">
       <c r="A60" s="34" t="inlineStr">
@@ -2250,6 +2310,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="34" customHeight="1">
       <c r="A61" s="34" t="inlineStr">
@@ -2277,6 +2342,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="34" customHeight="1">
       <c r="A62" s="34" t="inlineStr">
@@ -2304,6 +2374,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="34" customHeight="1">
       <c r="A63" s="34" t="inlineStr">
@@ -2331,6 +2406,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="34" customHeight="1">
       <c r="A64" s="34" t="inlineStr">
@@ -2358,6 +2438,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="34" customHeight="1">
       <c r="A65" s="34" t="inlineStr">
@@ -2385,6 +2470,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="34" customHeight="1">
       <c r="A66" s="34" t="inlineStr">
@@ -2412,6 +2502,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="34" customHeight="1">
       <c r="A67" s="34" t="inlineStr">
@@ -2439,6 +2534,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="34" customHeight="1">
       <c r="A68" s="34" t="inlineStr">
@@ -2466,6 +2566,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="34" customHeight="1">
       <c r="A69" s="34" t="inlineStr">
@@ -2493,6 +2598,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="34" customHeight="1">
       <c r="A70" s="34" t="inlineStr">
@@ -2520,6 +2630,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="34" customHeight="1">
       <c r="A71" s="34" t="inlineStr">
@@ -2547,6 +2662,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="34" customHeight="1">
       <c r="A72" s="34" t="inlineStr">
@@ -2574,6 +2694,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="34" customHeight="1">
       <c r="A73" s="34" t="inlineStr">
@@ -2601,6 +2726,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="34" customHeight="1">
       <c r="A74" s="34" t="inlineStr">
@@ -2628,6 +2758,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="34" customHeight="1">
       <c r="A75" s="34" t="inlineStr">
@@ -2655,6 +2790,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="34" customHeight="1">
       <c r="A76" s="34" t="inlineStr">
@@ -2682,6 +2822,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="34" customHeight="1">
       <c r="A77" s="34" t="inlineStr">
@@ -2709,6 +2854,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="34" customHeight="1">
       <c r="A78" s="34" t="inlineStr">
@@ -2736,6 +2886,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="34" customHeight="1">
       <c r="A79" s="34" t="inlineStr">
@@ -2763,6 +2918,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="34" customHeight="1">
       <c r="A80" s="34" t="inlineStr">
@@ -2790,6 +2950,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="34" customHeight="1">
       <c r="A81" s="34" t="inlineStr">
@@ -2817,6 +2982,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="34" customHeight="1">
       <c r="A82" s="34" t="inlineStr">
@@ -2844,6 +3014,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="34" customHeight="1">
       <c r="A83" s="34" t="inlineStr">
@@ -2871,6 +3046,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="34" customHeight="1">
       <c r="A84" s="34" t="inlineStr">
@@ -2898,6 +3078,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="34" customHeight="1">
       <c r="A85" s="34" t="inlineStr">
@@ -2925,6 +3110,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="34" customHeight="1">
       <c r="A86" s="34" t="inlineStr">
@@ -2952,6 +3142,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="34" customHeight="1">
       <c r="A87" s="34" t="inlineStr">
@@ -2979,6 +3174,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="34" customHeight="1">
       <c r="A88" s="34" t="inlineStr">
@@ -3006,6 +3206,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="34" customHeight="1">
       <c r="A89" s="34" t="inlineStr">
@@ -3033,6 +3238,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="34" customHeight="1">
       <c r="A90" s="34" t="inlineStr">
@@ -3060,6 +3270,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="34" customHeight="1">
       <c r="A91" s="34" t="inlineStr">
@@ -3087,6 +3302,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="34" customHeight="1">
       <c r="A92" s="34" t="inlineStr">
@@ -3114,6 +3334,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="34" customHeight="1">
       <c r="A93" s="34" t="inlineStr">
@@ -3141,6 +3366,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="34" customHeight="1">
       <c r="A94" s="34" t="inlineStr">
@@ -3168,6 +3398,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="34" customHeight="1">
       <c r="A95" s="34" t="inlineStr">
@@ -3195,6 +3430,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="34" customHeight="1">
       <c r="A96" s="34" t="inlineStr">
@@ -3222,6 +3462,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="34" customHeight="1">
       <c r="A97" s="34" t="inlineStr">
@@ -3249,6 +3494,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="34" customHeight="1">
       <c r="A98" s="34" t="inlineStr">
@@ -3276,6 +3526,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="34" customHeight="1">
       <c r="A99" s="34" t="inlineStr">
@@ -3303,6 +3558,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="34" customHeight="1">
       <c r="A100" s="34" t="inlineStr">
@@ -3330,6 +3590,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="34" customHeight="1">
       <c r="A101" s="34" t="inlineStr">
@@ -3357,6 +3622,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="34" customHeight="1">
       <c r="A102" s="34" t="inlineStr">
@@ -3384,6 +3654,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="34" customHeight="1">
       <c r="A103" s="34" t="inlineStr">
@@ -3411,6 +3686,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="34" customHeight="1">
       <c r="A104" s="34" t="inlineStr">
@@ -3438,6 +3718,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="34" customHeight="1">
       <c r="A105" s="34" t="inlineStr">
@@ -3465,6 +3750,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="34" customHeight="1">
       <c r="A106" s="34" t="inlineStr">
@@ -3492,6 +3782,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="34" customHeight="1">
       <c r="A107" s="34" t="inlineStr">
@@ -3519,6 +3814,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="34" customHeight="1">
       <c r="A108" s="34" t="inlineStr">
@@ -3546,6 +3846,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="34" customHeight="1">
       <c r="A109" s="34" t="inlineStr">
@@ -3573,6 +3878,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="34" customHeight="1">
       <c r="A110" s="34" t="inlineStr">
@@ -3600,6 +3910,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="34" customHeight="1">
       <c r="A111" s="34" t="inlineStr">
@@ -3627,6 +3942,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="34" customHeight="1">
       <c r="A112" s="34" t="inlineStr">
@@ -3654,6 +3974,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="34" customHeight="1">
       <c r="A113" s="34" t="inlineStr">
@@ -3681,6 +4006,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="34" customHeight="1">
       <c r="A114" s="34" t="inlineStr">
@@ -3708,6 +4038,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="34" customHeight="1">
       <c r="A115" s="34" t="inlineStr">
@@ -3735,6 +4070,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="34" customHeight="1">
       <c r="A116" s="34" t="inlineStr">
@@ -3762,6 +4102,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="34" customHeight="1">
       <c r="A117" s="34" t="inlineStr">
@@ -3789,6 +4134,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="34" customHeight="1">
       <c r="A118" s="34" t="inlineStr">
@@ -3816,6 +4166,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="34" customHeight="1">
       <c r="A119" s="34" t="inlineStr">
@@ -3843,6 +4198,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="34" customHeight="1">
       <c r="A120" s="34" t="inlineStr">
@@ -3870,6 +4230,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="34" customHeight="1">
       <c r="A121" s="34" t="inlineStr">
@@ -3897,6 +4262,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="34" customHeight="1">
       <c r="A122" s="34" t="inlineStr">
@@ -3924,6 +4294,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="34" customHeight="1">
       <c r="A123" s="34" t="inlineStr">
@@ -3951,6 +4326,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="34" customHeight="1">
       <c r="A124" s="34" t="inlineStr">
@@ -3978,6 +4358,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="34" customHeight="1">
       <c r="A125" s="34" t="inlineStr">
@@ -4005,6 +4390,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="34" customHeight="1">
       <c r="A126" s="34" t="inlineStr">
@@ -4032,6 +4422,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="34" customHeight="1">
       <c r="A127" s="34" t="inlineStr">
@@ -4059,6 +4454,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="34" customHeight="1">
       <c r="A128" s="34" t="inlineStr">
@@ -4086,6 +4486,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="34" customHeight="1">
       <c r="A129" s="34" t="inlineStr">
@@ -4113,6 +4518,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="34" customHeight="1">
       <c r="A130" s="34" t="inlineStr">
@@ -4140,6 +4550,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="34" customHeight="1">
       <c r="A131" s="34" t="inlineStr">
@@ -4167,6 +4582,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="34" customHeight="1">
       <c r="A132" s="34" t="inlineStr">
@@ -4194,6 +4614,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="34" customHeight="1">
       <c r="A133" s="34" t="inlineStr">
@@ -4221,6 +4646,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="34" customHeight="1">
       <c r="A134" s="34" t="inlineStr">
@@ -4248,6 +4678,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="34" customHeight="1">
       <c r="A135" s="34" t="inlineStr">
@@ -4275,6 +4710,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="34" customHeight="1">
       <c r="A136" s="34" t="inlineStr">
@@ -4302,6 +4742,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="34" customHeight="1">
       <c r="A137" s="34" t="inlineStr">
@@ -4329,6 +4774,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="34" customHeight="1">
       <c r="A138" s="34" t="inlineStr">
@@ -4356,6 +4806,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="34" customHeight="1">
       <c r="A139" s="34" t="inlineStr">
@@ -4383,6 +4838,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="34" customHeight="1">
       <c r="A140" s="34" t="inlineStr">
@@ -4410,6 +4870,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="34" customHeight="1">
       <c r="A141" s="34" t="inlineStr">
@@ -4437,6 +4902,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="34" customHeight="1">
       <c r="A142" s="34" t="inlineStr">
@@ -4464,6 +4934,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="34" customHeight="1">
       <c r="A143" s="34" t="inlineStr">
@@ -4491,6 +4966,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="34" customHeight="1">
       <c r="A144" s="34" t="inlineStr">
@@ -4518,6 +4998,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="34" customHeight="1">
       <c r="A145" s="34" t="inlineStr">
@@ -4545,6 +5030,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="34" customHeight="1">
       <c r="A146" s="34" t="inlineStr">
@@ -4572,6 +5062,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="34" customHeight="1">
       <c r="A147" s="34" t="inlineStr">
@@ -4599,6 +5094,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="34" customHeight="1">
       <c r="A148" s="34" t="inlineStr">
@@ -4626,6 +5126,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="34" customHeight="1">
       <c r="A149" s="34" t="inlineStr">
@@ -4653,6 +5158,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="34" customHeight="1">
       <c r="A150" s="34" t="inlineStr">
@@ -4680,6 +5190,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="34" customHeight="1">
       <c r="A151" s="34" t="inlineStr">
@@ -4707,6 +5222,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="34" customHeight="1">
       <c r="A152" s="34" t="inlineStr">
@@ -4734,6 +5254,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="34" customHeight="1">
       <c r="A153" s="34" t="inlineStr">
@@ -4761,6 +5286,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="34" customHeight="1">
       <c r="A154" s="34" t="inlineStr">
@@ -4788,6 +5318,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="34" customHeight="1">
       <c r="A155" s="34" t="inlineStr">
@@ -4815,6 +5350,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="34" customHeight="1">
       <c r="A156" s="34" t="inlineStr">
@@ -4842,6 +5382,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="34" customHeight="1">
       <c r="A157" s="34" t="inlineStr">
@@ -4869,6 +5414,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="34" customHeight="1">
       <c r="A158" s="34" t="inlineStr">
@@ -4896,6 +5446,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="159" ht="34" customHeight="1">
       <c r="A159" s="34" t="inlineStr">
@@ -4923,6 +5478,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="160" ht="34" customHeight="1">
       <c r="A160" s="34" t="inlineStr">
@@ -4950,6 +5510,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="34" customHeight="1">
       <c r="A161" s="34" t="inlineStr">
@@ -4977,6 +5542,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="34" customHeight="1">
       <c r="A162" s="34" t="inlineStr">
@@ -5004,6 +5574,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="34" customHeight="1">
       <c r="A163" s="34" t="inlineStr">
@@ -5031,6 +5606,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="34" customHeight="1">
       <c r="A164" s="34" t="inlineStr">
@@ -5058,6 +5638,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="34" customHeight="1">
       <c r="A165" s="34" t="inlineStr">
@@ -5085,6 +5670,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="166" ht="34" customHeight="1">
       <c r="A166" s="34" t="inlineStr">
@@ -5112,6 +5702,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="167" ht="34" customHeight="1">
       <c r="A167" s="34" t="inlineStr">
@@ -5139,6 +5734,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="34" customHeight="1">
       <c r="A168" s="34" t="inlineStr">
@@ -5166,6 +5766,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="169" ht="34" customHeight="1">
       <c r="A169" s="34" t="inlineStr">
@@ -5193,6 +5798,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="34" customHeight="1">
       <c r="A170" s="34" t="inlineStr">
@@ -5220,6 +5830,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="171" ht="34" customHeight="1">
       <c r="A171" s="34" t="inlineStr">
@@ -5247,6 +5862,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="34" customHeight="1">
       <c r="A172" s="34" t="inlineStr">
@@ -5274,6 +5894,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="34" customHeight="1">
       <c r="A173" s="34" t="inlineStr">
@@ -5301,6 +5926,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="174" ht="34" customHeight="1">
       <c r="A174" s="34" t="inlineStr">
@@ -5328,6 +5958,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="34" customHeight="1">
       <c r="A175" s="34" t="inlineStr">
@@ -5355,6 +5990,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="176" ht="34" customHeight="1">
       <c r="A176" s="34" t="inlineStr">
@@ -5382,6 +6022,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="177" ht="34" customHeight="1">
       <c r="A177" s="34" t="inlineStr">
@@ -5409,6 +6054,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="178" ht="34" customHeight="1">
       <c r="A178" s="34" t="inlineStr">
@@ -5436,6 +6086,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="179" ht="34" customHeight="1">
       <c r="A179" s="34" t="inlineStr">
@@ -5463,6 +6118,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="180" ht="34" customHeight="1">
       <c r="A180" s="34" t="inlineStr">
@@ -5490,6 +6150,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="181" ht="34" customHeight="1">
       <c r="A181" s="34" t="inlineStr">
@@ -5517,6 +6182,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="34" customHeight="1">
       <c r="A182" s="34" t="inlineStr">
@@ -5544,6 +6214,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="183" ht="34" customHeight="1">
       <c r="A183" s="34" t="inlineStr">
@@ -5571,6 +6246,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="34" customHeight="1">
       <c r="A184" s="34" t="inlineStr">
@@ -5598,6 +6278,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="185" ht="34" customHeight="1">
       <c r="A185" s="34" t="inlineStr">
@@ -5625,6 +6310,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="186" ht="34" customHeight="1">
       <c r="A186" s="34" t="inlineStr">
@@ -5652,6 +6342,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="187" ht="34" customHeight="1">
       <c r="A187" s="34" t="inlineStr">
@@ -5679,6 +6374,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="188" ht="34" customHeight="1">
       <c r="A188" s="34" t="inlineStr">
@@ -5706,6 +6406,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="189" ht="34" customHeight="1">
       <c r="A189" s="34" t="inlineStr">
@@ -5733,6 +6438,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="190" ht="34" customHeight="1">
       <c r="A190" s="34" t="inlineStr">
@@ -5760,6 +6470,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="191" ht="34" customHeight="1">
       <c r="A191" s="34" t="inlineStr">
@@ -5787,6 +6502,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="192" ht="34" customHeight="1">
       <c r="A192" s="34" t="inlineStr">
@@ -5814,6 +6534,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="193" ht="34" customHeight="1">
       <c r="A193" s="34" t="inlineStr">
@@ -5841,6 +6566,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="194" ht="34" customHeight="1">
       <c r="A194" s="34" t="inlineStr">
@@ -5868,6 +6598,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="195" ht="34" customHeight="1">
       <c r="A195" s="34" t="inlineStr">
@@ -5895,6 +6630,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="196" ht="34" customHeight="1">
       <c r="A196" s="34" t="inlineStr">
@@ -5922,6 +6662,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="197" ht="34" customHeight="1">
       <c r="A197" s="34" t="inlineStr">
@@ -5949,6 +6694,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="198" ht="34" customHeight="1">
       <c r="A198" s="34" t="inlineStr">
@@ -5976,6 +6726,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="199" ht="34" customHeight="1">
       <c r="A199" s="34" t="inlineStr">
@@ -6003,6 +6758,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="200" ht="34" customHeight="1">
       <c r="A200" s="34" t="inlineStr">
@@ -6030,6 +6790,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="201" ht="34" customHeight="1">
       <c r="A201" s="34" t="inlineStr">
@@ -6057,6 +6822,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="202" ht="34" customHeight="1">
       <c r="A202" s="34" t="inlineStr">
@@ -6084,6 +6854,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="203" ht="34" customHeight="1">
       <c r="A203" s="34" t="inlineStr">
@@ -6111,6 +6886,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="204" ht="34" customHeight="1">
       <c r="A204" s="34" t="inlineStr">
@@ -6138,6 +6918,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="205" ht="34" customHeight="1">
       <c r="A205" s="34" t="inlineStr">
@@ -6165,6 +6950,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="206" ht="34" customHeight="1">
       <c r="A206" s="34" t="inlineStr">
@@ -6192,6 +6982,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="207" ht="34" customHeight="1">
       <c r="A207" s="34" t="inlineStr">
@@ -6219,6 +7014,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="208" ht="34" customHeight="1">
       <c r="A208" s="34" t="inlineStr">
@@ -6246,6 +7046,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="209" ht="34" customHeight="1">
       <c r="A209" s="34" t="inlineStr">
@@ -6273,6 +7078,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="210" ht="34" customHeight="1">
       <c r="A210" s="34" t="inlineStr">
@@ -6300,6 +7110,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="211" ht="34" customHeight="1">
       <c r="A211" s="34" t="inlineStr">
@@ -6327,6 +7142,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="212" ht="34" customHeight="1">
       <c r="A212" s="34" t="inlineStr">
@@ -6354,6 +7174,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="213" ht="34" customHeight="1">
       <c r="A213" s="34" t="inlineStr">
@@ -6381,6 +7206,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="214" ht="34" customHeight="1">
       <c r="A214" s="34" t="inlineStr">
@@ -6408,6 +7238,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="215" ht="34" customHeight="1">
       <c r="A215" s="34" t="inlineStr">
@@ -6435,6 +7270,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="216" ht="34" customHeight="1">
       <c r="A216" s="34" t="inlineStr">
@@ -6462,6 +7302,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="217" ht="34" customHeight="1">
       <c r="A217" s="34" t="inlineStr">
@@ -6489,6 +7334,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="218" ht="34" customHeight="1">
       <c r="A218" s="34" t="inlineStr">
@@ -6516,6 +7366,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="219" ht="34" customHeight="1">
       <c r="A219" s="34" t="inlineStr">
@@ -6543,6 +7398,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="220" ht="34" customHeight="1">
       <c r="A220" s="34" t="inlineStr">
@@ -6570,6 +7430,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="221" ht="34" customHeight="1">
       <c r="A221" s="34" t="inlineStr">
@@ -6597,6 +7462,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="222" ht="34" customHeight="1">
       <c r="A222" s="34" t="inlineStr">
@@ -6624,6 +7494,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="223" ht="34" customHeight="1">
       <c r="A223" s="34" t="inlineStr">
@@ -6651,6 +7526,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="224" ht="34" customHeight="1">
       <c r="A224" s="34" t="inlineStr">
@@ -6678,6 +7558,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="225" ht="34" customHeight="1">
       <c r="A225" s="34" t="inlineStr">
@@ -6705,6 +7590,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="226" ht="34" customHeight="1">
       <c r="A226" s="34" t="inlineStr">
@@ -6732,6 +7622,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="227" ht="34" customHeight="1">
       <c r="A227" s="34" t="inlineStr">
@@ -6759,6 +7654,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="228" ht="34" customHeight="1">
       <c r="A228" s="34" t="inlineStr">
@@ -6786,6 +7686,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="229" ht="34" customHeight="1">
       <c r="A229" s="34" t="inlineStr">
@@ -6813,6 +7718,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="230" ht="34" customHeight="1">
       <c r="A230" s="34" t="inlineStr">
@@ -6840,6 +7750,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="231" ht="34" customHeight="1">
       <c r="A231" s="34" t="inlineStr">
@@ -6867,6 +7782,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="232" ht="34" customHeight="1">
       <c r="A232" s="34" t="inlineStr">
@@ -6894,6 +7814,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="233" ht="34" customHeight="1">
       <c r="A233" s="34" t="inlineStr">
@@ -6921,6 +7846,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="234" ht="34" customHeight="1">
       <c r="A234" s="34" t="inlineStr">
@@ -6948,6 +7878,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="235" ht="34" customHeight="1">
       <c r="A235" s="34" t="inlineStr">
@@ -6975,6 +7910,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="236" ht="34" customHeight="1">
       <c r="A236" s="34" t="inlineStr">
@@ -7002,6 +7942,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="237" ht="34" customHeight="1">
       <c r="A237" s="34" t="inlineStr">
@@ -7029,6 +7974,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="238" ht="34" customHeight="1">
       <c r="A238" s="34" t="inlineStr">
@@ -7056,6 +8006,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="239" ht="34" customHeight="1">
       <c r="A239" s="34" t="inlineStr">
@@ -7083,6 +8038,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="240" ht="34" customHeight="1">
       <c r="A240" s="34" t="inlineStr">
@@ -7110,6 +8070,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="241" ht="34" customHeight="1">
       <c r="A241" s="34" t="inlineStr">
@@ -7137,6 +8102,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="242" ht="34" customHeight="1">
       <c r="A242" s="34" t="inlineStr">
@@ -7164,6 +8134,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="243" ht="34" customHeight="1">
       <c r="A243" s="34" t="inlineStr">
@@ -7191,6 +8166,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="244" ht="34" customHeight="1">
       <c r="A244" s="34" t="inlineStr">
@@ -7218,6 +8198,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="245" ht="34" customHeight="1">
       <c r="A245" s="34" t="inlineStr">
@@ -7245,6 +8230,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="246" ht="34" customHeight="1">
       <c r="A246" s="34" t="inlineStr">
@@ -7272,6 +8262,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="247" ht="34" customHeight="1">
       <c r="A247" s="34" t="inlineStr">
@@ -7299,6 +8294,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="248" ht="34" customHeight="1">
       <c r="A248" s="34" t="inlineStr">
@@ -7326,6 +8326,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="249" ht="34" customHeight="1">
       <c r="A249" s="34" t="inlineStr">
@@ -7353,6 +8358,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="250" ht="34" customHeight="1">
       <c r="A250" s="34" t="inlineStr">
@@ -7380,6 +8390,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="251" ht="34" customHeight="1">
       <c r="A251" s="34" t="inlineStr">
@@ -7407,6 +8422,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="252" ht="34" customHeight="1">
       <c r="A252" s="34" t="inlineStr">
@@ -7434,6 +8454,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="253" ht="34" customHeight="1">
       <c r="A253" s="34" t="inlineStr">
@@ -7461,6 +8486,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="254" ht="34" customHeight="1">
       <c r="A254" s="34" t="inlineStr">
@@ -7488,6 +8518,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="255" ht="34" customHeight="1">
       <c r="A255" s="34" t="inlineStr">
@@ -7515,6 +8550,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="256" ht="34" customHeight="1">
       <c r="A256" s="34" t="inlineStr">
@@ -7542,6 +8582,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="257" ht="34" customHeight="1">
       <c r="A257" s="34" t="inlineStr">
@@ -7569,6 +8614,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="258" ht="34" customHeight="1">
       <c r="A258" s="34" t="inlineStr">
@@ -7596,6 +8646,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="259" ht="34" customHeight="1">
       <c r="A259" s="34" t="inlineStr">
@@ -7623,6 +8678,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="260" ht="34" customHeight="1">
       <c r="A260" s="34" t="inlineStr">
@@ -7650,6 +8710,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="261" ht="34" customHeight="1">
       <c r="A261" s="34" t="inlineStr">
@@ -7677,6 +8742,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="262" ht="34" customHeight="1">
       <c r="A262" s="34" t="inlineStr">
@@ -7704,6 +8774,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="263" ht="34" customHeight="1">
       <c r="A263" s="34" t="inlineStr">
@@ -7731,6 +8806,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="264" ht="34" customHeight="1">
       <c r="A264" s="34" t="inlineStr">
@@ -7758,6 +8838,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="265" ht="34" customHeight="1">
       <c r="A265" s="34" t="inlineStr">
@@ -7785,6 +8870,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="266" ht="34" customHeight="1">
       <c r="A266" s="34" t="inlineStr">
@@ -7812,6 +8902,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="267" ht="34" customHeight="1">
       <c r="A267" s="34" t="inlineStr">
@@ -7839,6 +8934,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="268" ht="34" customHeight="1">
       <c r="A268" s="34" t="inlineStr">
@@ -7866,6 +8966,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="269" ht="34" customHeight="1">
       <c r="A269" s="34" t="inlineStr">
@@ -7893,6 +8998,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="270" ht="34" customHeight="1">
       <c r="A270" s="34" t="inlineStr">
@@ -7920,6 +9030,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="271" ht="34" customHeight="1">
       <c r="A271" s="34" t="inlineStr">
@@ -7947,6 +9062,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="272" ht="34" customHeight="1">
       <c r="A272" s="34" t="inlineStr">
@@ -7974,6 +9094,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="273" ht="34" customHeight="1">
       <c r="A273" s="34" t="inlineStr">
@@ -8001,6 +9126,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="274" ht="34" customHeight="1">
       <c r="A274" s="34" t="inlineStr">
@@ -8028,6 +9158,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="275" ht="34" customHeight="1">
       <c r="A275" s="34" t="inlineStr">
@@ -8055,6 +9190,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="276" ht="34" customHeight="1">
       <c r="A276" s="34" t="inlineStr">
@@ -8082,6 +9222,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="277" ht="34" customHeight="1">
       <c r="A277" s="34" t="inlineStr">
@@ -8109,6 +9254,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="278" ht="34" customHeight="1">
       <c r="A278" s="34" t="inlineStr">
@@ -8136,6 +9286,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="279" ht="34" customHeight="1">
       <c r="A279" s="34" t="inlineStr">
@@ -8163,6 +9318,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="280" ht="34" customHeight="1">
       <c r="A280" s="34" t="inlineStr">
@@ -8190,6 +9350,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="281" ht="34" customHeight="1">
       <c r="A281" s="34" t="inlineStr">
@@ -8217,6 +9382,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="282" ht="34" customHeight="1">
       <c r="A282" s="34" t="inlineStr">
@@ -8244,6 +9414,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="283" ht="34" customHeight="1">
       <c r="A283" s="34" t="inlineStr">
@@ -8271,6 +9446,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="284" ht="34" customHeight="1">
       <c r="A284" s="34" t="inlineStr">
@@ -8298,6 +9478,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="285" ht="34" customHeight="1">
       <c r="A285" s="34" t="inlineStr">
@@ -8325,6 +9510,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="286" ht="34" customHeight="1">
       <c r="A286" s="34" t="inlineStr">
@@ -8352,6 +9542,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="287" ht="34" customHeight="1">
       <c r="A287" s="34" t="inlineStr">
@@ -8379,6 +9574,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="288" ht="34" customHeight="1">
       <c r="A288" s="34" t="inlineStr">
@@ -8406,6 +9606,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="289" ht="34" customHeight="1">
       <c r="A289" s="34" t="inlineStr">
@@ -8433,6 +9638,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="290" ht="34" customHeight="1">
       <c r="A290" s="34" t="inlineStr">
@@ -8460,6 +9670,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="291" ht="34" customHeight="1">
       <c r="A291" s="34" t="inlineStr">
@@ -8487,6 +9702,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="292" ht="34" customHeight="1">
       <c r="A292" s="34" t="inlineStr">
@@ -8514,6 +9734,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="293" ht="34" customHeight="1">
       <c r="A293" s="34" t="inlineStr">
@@ -8541,6 +9766,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="294" ht="34" customHeight="1">
       <c r="A294" s="34" t="inlineStr">
@@ -8568,6 +9798,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="295" ht="34" customHeight="1">
       <c r="A295" s="34" t="inlineStr">
@@ -8595,6 +9830,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="296" ht="34" customHeight="1">
       <c r="A296" s="34" t="inlineStr">
@@ -8622,6 +9862,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="297" ht="34" customHeight="1">
       <c r="A297" s="34" t="inlineStr">
@@ -8649,6 +9894,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="298" ht="34" customHeight="1">
       <c r="A298" s="34" t="inlineStr">
@@ -8676,6 +9926,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="299" ht="34" customHeight="1">
       <c r="A299" s="34" t="inlineStr">
@@ -8703,6 +9958,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="300" ht="34" customHeight="1">
       <c r="A300" s="34" t="inlineStr">
@@ -8730,6 +9990,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="301" ht="34" customHeight="1">
       <c r="A301" s="34" t="inlineStr">
@@ -8757,6 +10022,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="302" ht="34" customHeight="1">
       <c r="A302" s="34" t="inlineStr">
@@ -8784,6 +10054,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="303" ht="34" customHeight="1">
       <c r="A303" s="34" t="inlineStr">
@@ -8811,6 +10086,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="304" ht="34" customHeight="1">
       <c r="A304" s="34" t="inlineStr">
@@ -8838,6 +10118,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="305" ht="34" customHeight="1">
       <c r="A305" s="34" t="inlineStr">
@@ -8865,6 +10150,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="306" ht="34" customHeight="1">
       <c r="A306" s="34" t="inlineStr">
@@ -8892,6 +10182,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="307" ht="34" customHeight="1">
       <c r="A307" s="34" t="inlineStr">
@@ -8919,6 +10214,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="308" ht="34" customHeight="1">
       <c r="A308" s="34" t="inlineStr">
@@ -8946,6 +10246,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="309" ht="34" customHeight="1">
       <c r="A309" s="34" t="inlineStr">
@@ -8973,6 +10278,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="310" ht="34" customHeight="1">
       <c r="A310" s="34" t="inlineStr">
@@ -9000,6 +10310,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="311" ht="34" customHeight="1">
       <c r="A311" s="34" t="inlineStr">
@@ -9027,6 +10342,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="312" ht="34" customHeight="1">
       <c r="A312" s="34" t="inlineStr">
@@ -9054,6 +10374,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="313" ht="34" customHeight="1">
       <c r="A313" s="34" t="inlineStr">
@@ -9081,6 +10406,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="314" ht="34" customHeight="1">
       <c r="A314" s="34" t="inlineStr">
@@ -9108,6 +10438,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="315" ht="34" customHeight="1">
       <c r="A315" s="34" t="inlineStr">
@@ -9135,6 +10470,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="316" ht="34" customHeight="1">
       <c r="A316" s="34" t="inlineStr">
@@ -9162,6 +10502,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="317" ht="34" customHeight="1">
       <c r="A317" s="34" t="inlineStr">
@@ -9189,6 +10534,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="318" ht="34" customHeight="1">
       <c r="A318" s="34" t="inlineStr">
@@ -9216,6 +10566,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="319" ht="34" customHeight="1">
       <c r="A319" s="34" t="inlineStr">
@@ -9243,6 +10598,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="320" ht="34" customHeight="1">
       <c r="A320" s="34" t="inlineStr">
@@ -9270,6 +10630,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="321" ht="34" customHeight="1">
       <c r="A321" s="34" t="inlineStr">
@@ -9297,6 +10662,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="322" ht="34" customHeight="1">
       <c r="A322" s="34" t="inlineStr">
@@ -9324,6 +10694,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="323" ht="34" customHeight="1">
       <c r="A323" s="34" t="inlineStr">
@@ -9351,6 +10726,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="324" ht="34" customHeight="1">
       <c r="A324" s="34" t="inlineStr">
@@ -9378,6 +10758,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="325" ht="34" customHeight="1">
       <c r="A325" s="34" t="inlineStr">
@@ -9405,6 +10790,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="326" ht="34" customHeight="1">
       <c r="A326" s="34" t="inlineStr">
@@ -9432,6 +10822,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="327" ht="34" customHeight="1">
       <c r="A327" s="34" t="inlineStr">
@@ -9459,6 +10854,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="328" ht="34" customHeight="1">
       <c r="A328" s="34" t="inlineStr">
@@ -9486,6 +10886,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="329" ht="34" customHeight="1">
       <c r="A329" s="34" t="inlineStr">
@@ -9513,6 +10918,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="330" ht="34" customHeight="1">
       <c r="A330" s="34" t="inlineStr">
@@ -9540,6 +10950,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="331" ht="34" customHeight="1">
       <c r="A331" s="34" t="inlineStr">
@@ -9567,6 +10982,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="332" ht="34" customHeight="1">
       <c r="A332" s="34" t="inlineStr">
@@ -9594,6 +11014,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="333" ht="34" customHeight="1">
       <c r="A333" s="34" t="inlineStr">
@@ -9621,6 +11046,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="334" ht="34" customHeight="1">
       <c r="A334" s="34" t="inlineStr">
@@ -9648,6 +11078,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="335" ht="34" customHeight="1">
       <c r="A335" s="34" t="inlineStr">
@@ -9675,6 +11110,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="336" ht="34" customHeight="1">
       <c r="A336" s="34" t="inlineStr">
@@ -9702,6 +11142,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="337" ht="34" customHeight="1">
       <c r="A337" s="34" t="inlineStr">
@@ -9729,6 +11174,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="338" ht="34" customHeight="1">
       <c r="A338" s="34" t="inlineStr">
@@ -9756,6 +11206,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="339" ht="34" customHeight="1">
       <c r="A339" s="34" t="inlineStr">
@@ -9783,6 +11238,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="340" ht="34" customHeight="1">
       <c r="A340" s="34" t="inlineStr">
@@ -9810,6 +11270,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="341" ht="34" customHeight="1">
       <c r="A341" s="34" t="inlineStr">
@@ -9837,6 +11302,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="342" ht="34" customHeight="1">
       <c r="A342" s="34" t="inlineStr">
@@ -9864,6 +11334,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="343" ht="34" customHeight="1">
       <c r="A343" s="34" t="inlineStr">
@@ -9891,6 +11366,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="344" ht="34" customHeight="1">
       <c r="A344" s="34" t="inlineStr">
@@ -9918,6 +11398,11 @@
           <t>☑</t>
         </is>
       </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="345" ht="34" customHeight="1">
       <c r="A345" s="34" t="inlineStr">
@@ -9945,6 +11430,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="346" ht="34" customHeight="1">
       <c r="A346" s="34" t="inlineStr">
@@ -9972,6 +11462,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="347" ht="34" customHeight="1">
       <c r="A347" s="34" t="inlineStr">
@@ -9999,6 +11494,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="348" ht="34" customHeight="1">
       <c r="A348" s="34" t="inlineStr">
@@ -10026,6 +11526,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="349" ht="34" customHeight="1">
       <c r="A349" s="34" t="inlineStr">
@@ -10053,6 +11558,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="350" ht="34" customHeight="1">
       <c r="A350" s="34" t="inlineStr">
@@ -10080,6 +11590,11 @@
           <t>☐</t>
         </is>
       </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
     </row>
     <row r="351" ht="34" customHeight="1">
       <c r="A351" s="34" t="inlineStr">
@@ -10105,6 +11620,11 @@
       <c r="E351" s="40" t="inlineStr">
         <is>
           <t>☐</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>

</xml_diff>